<commit_message>
feat: add specific widths to different columns in template excel file
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -354,6 +354,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="3" min="3" width="11"/>
+    <col customWidth="true" max="6" min="6" width="13"/>
+    <col customWidth="true" max="8" min="7" width="12"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
refactor: improve header style on template
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -56,15 +56,20 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB2B2B2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -72,12 +77,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="false">
+      <alignment/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -361,31 +383,31 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>